<commit_message>
Cek 1: pilihan tahap judul menjadi Yes/Yes-C1/Yes-C3/No; skrip kappa menerimanya
Claude-Session: https://claude.ai/code/session_01BPtQFpvpVz4zo6iW3nzWcR
</commit_message>
<xml_diff>
--- a/literature/scopus-2026-09/verifikasi/sampel_judul.xlsx
+++ b/literature/scopus-2026-09/verifikasi/sampel_judul.xlsx
@@ -528,7 +528,6 @@
       </c>
       <c r="G2" s="3" t="inlineStr"/>
       <c r="H2" s="4" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
       <c r="J2" s="3" t="inlineStr"/>
     </row>
     <row r="3">
@@ -562,7 +561,6 @@
       </c>
       <c r="G3" s="3" t="inlineStr"/>
       <c r="H3" s="4" t="inlineStr"/>
-      <c r="I3" t="inlineStr"/>
       <c r="J3" s="3" t="inlineStr"/>
     </row>
     <row r="4">
@@ -596,7 +594,6 @@
       </c>
       <c r="G4" s="3" t="inlineStr"/>
       <c r="H4" s="4" t="inlineStr"/>
-      <c r="I4" t="inlineStr"/>
       <c r="J4" s="3" t="inlineStr"/>
     </row>
     <row r="5">
@@ -630,7 +627,6 @@
       </c>
       <c r="G5" s="3" t="inlineStr"/>
       <c r="H5" s="4" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
       <c r="J5" s="3" t="inlineStr"/>
     </row>
     <row r="6">
@@ -664,7 +660,6 @@
       </c>
       <c r="G6" s="3" t="inlineStr"/>
       <c r="H6" s="4" t="inlineStr"/>
-      <c r="I6" t="inlineStr"/>
       <c r="J6" s="3" t="inlineStr"/>
     </row>
     <row r="7">
@@ -698,7 +693,6 @@
       </c>
       <c r="G7" s="3" t="inlineStr"/>
       <c r="H7" s="4" t="inlineStr"/>
-      <c r="I7" t="inlineStr"/>
       <c r="J7" s="3" t="inlineStr"/>
     </row>
     <row r="8">
@@ -732,7 +726,6 @@
       </c>
       <c r="G8" s="3" t="inlineStr"/>
       <c r="H8" s="4" t="inlineStr"/>
-      <c r="I8" t="inlineStr"/>
       <c r="J8" s="3" t="inlineStr"/>
     </row>
     <row r="9">
@@ -766,7 +759,6 @@
       </c>
       <c r="G9" s="3" t="inlineStr"/>
       <c r="H9" s="4" t="inlineStr"/>
-      <c r="I9" t="inlineStr"/>
       <c r="J9" s="3" t="inlineStr"/>
     </row>
     <row r="10">
@@ -800,7 +792,6 @@
       </c>
       <c r="G10" s="3" t="inlineStr"/>
       <c r="H10" s="4" t="inlineStr"/>
-      <c r="I10" t="inlineStr"/>
       <c r="J10" s="3" t="inlineStr"/>
     </row>
     <row r="11">
@@ -834,7 +825,6 @@
       </c>
       <c r="G11" s="3" t="inlineStr"/>
       <c r="H11" s="4" t="inlineStr"/>
-      <c r="I11" t="inlineStr"/>
       <c r="J11" s="3" t="inlineStr"/>
     </row>
     <row r="12">
@@ -868,7 +858,6 @@
       </c>
       <c r="G12" s="3" t="inlineStr"/>
       <c r="H12" s="4" t="inlineStr"/>
-      <c r="I12" t="inlineStr"/>
       <c r="J12" s="3" t="inlineStr"/>
     </row>
     <row r="13">
@@ -902,7 +891,6 @@
       </c>
       <c r="G13" s="3" t="inlineStr"/>
       <c r="H13" s="4" t="inlineStr"/>
-      <c r="I13" t="inlineStr"/>
       <c r="J13" s="3" t="inlineStr"/>
     </row>
     <row r="14">
@@ -936,7 +924,6 @@
       </c>
       <c r="G14" s="3" t="inlineStr"/>
       <c r="H14" s="4" t="inlineStr"/>
-      <c r="I14" t="inlineStr"/>
       <c r="J14" s="3" t="inlineStr"/>
     </row>
     <row r="15">
@@ -970,7 +957,6 @@
       </c>
       <c r="G15" s="3" t="inlineStr"/>
       <c r="H15" s="4" t="inlineStr"/>
-      <c r="I15" t="inlineStr"/>
       <c r="J15" s="3" t="inlineStr"/>
     </row>
     <row r="16">
@@ -1004,7 +990,6 @@
       </c>
       <c r="G16" s="3" t="inlineStr"/>
       <c r="H16" s="4" t="inlineStr"/>
-      <c r="I16" t="inlineStr"/>
       <c r="J16" s="3" t="inlineStr"/>
     </row>
     <row r="17">
@@ -1038,7 +1023,6 @@
       </c>
       <c r="G17" s="3" t="inlineStr"/>
       <c r="H17" s="4" t="inlineStr"/>
-      <c r="I17" t="inlineStr"/>
       <c r="J17" s="3" t="inlineStr"/>
     </row>
     <row r="18">
@@ -1072,7 +1056,6 @@
       </c>
       <c r="G18" s="3" t="inlineStr"/>
       <c r="H18" s="4" t="inlineStr"/>
-      <c r="I18" t="inlineStr"/>
       <c r="J18" s="3" t="inlineStr"/>
     </row>
     <row r="19">
@@ -1106,7 +1089,6 @@
       </c>
       <c r="G19" s="3" t="inlineStr"/>
       <c r="H19" s="4" t="inlineStr"/>
-      <c r="I19" t="inlineStr"/>
       <c r="J19" s="3" t="inlineStr"/>
     </row>
     <row r="20">
@@ -1140,7 +1122,6 @@
       </c>
       <c r="G20" s="3" t="inlineStr"/>
       <c r="H20" s="4" t="inlineStr"/>
-      <c r="I20" t="inlineStr"/>
       <c r="J20" s="3" t="inlineStr"/>
     </row>
     <row r="21">
@@ -1174,7 +1155,6 @@
       </c>
       <c r="G21" s="3" t="inlineStr"/>
       <c r="H21" s="4" t="inlineStr"/>
-      <c r="I21" t="inlineStr"/>
       <c r="J21" s="3" t="inlineStr"/>
     </row>
     <row r="22">
@@ -1208,7 +1188,6 @@
       </c>
       <c r="G22" s="3" t="inlineStr"/>
       <c r="H22" s="4" t="inlineStr"/>
-      <c r="I22" t="inlineStr"/>
       <c r="J22" s="3" t="inlineStr"/>
     </row>
     <row r="23">
@@ -1242,7 +1221,6 @@
       </c>
       <c r="G23" s="3" t="inlineStr"/>
       <c r="H23" s="4" t="inlineStr"/>
-      <c r="I23" t="inlineStr"/>
       <c r="J23" s="3" t="inlineStr"/>
     </row>
     <row r="24">
@@ -1276,7 +1254,6 @@
       </c>
       <c r="G24" s="3" t="inlineStr"/>
       <c r="H24" s="4" t="inlineStr"/>
-      <c r="I24" t="inlineStr"/>
       <c r="J24" s="3" t="inlineStr"/>
     </row>
     <row r="25">
@@ -1310,7 +1287,6 @@
       </c>
       <c r="G25" s="3" t="inlineStr"/>
       <c r="H25" s="4" t="inlineStr"/>
-      <c r="I25" t="inlineStr"/>
       <c r="J25" s="3" t="inlineStr"/>
     </row>
     <row r="26">
@@ -1344,7 +1320,6 @@
       </c>
       <c r="G26" s="3" t="inlineStr"/>
       <c r="H26" s="4" t="inlineStr"/>
-      <c r="I26" t="inlineStr"/>
       <c r="J26" s="3" t="inlineStr"/>
     </row>
     <row r="27">
@@ -1378,7 +1353,6 @@
       </c>
       <c r="G27" s="3" t="inlineStr"/>
       <c r="H27" s="4" t="inlineStr"/>
-      <c r="I27" t="inlineStr"/>
       <c r="J27" s="3" t="inlineStr"/>
     </row>
     <row r="28">
@@ -1412,7 +1386,6 @@
       </c>
       <c r="G28" s="3" t="inlineStr"/>
       <c r="H28" s="4" t="inlineStr"/>
-      <c r="I28" t="inlineStr"/>
       <c r="J28" s="3" t="inlineStr"/>
     </row>
     <row r="29">
@@ -1446,7 +1419,6 @@
       </c>
       <c r="G29" s="3" t="inlineStr"/>
       <c r="H29" s="4" t="inlineStr"/>
-      <c r="I29" t="inlineStr"/>
       <c r="J29" s="3" t="inlineStr"/>
     </row>
     <row r="30">
@@ -1480,7 +1452,6 @@
       </c>
       <c r="G30" s="3" t="inlineStr"/>
       <c r="H30" s="4" t="inlineStr"/>
-      <c r="I30" t="inlineStr"/>
       <c r="J30" s="3" t="inlineStr"/>
     </row>
     <row r="31">
@@ -1514,7 +1485,6 @@
       </c>
       <c r="G31" s="3" t="inlineStr"/>
       <c r="H31" s="4" t="inlineStr"/>
-      <c r="I31" t="inlineStr"/>
       <c r="J31" s="3" t="inlineStr"/>
     </row>
     <row r="32">
@@ -1548,7 +1518,6 @@
       </c>
       <c r="G32" s="3" t="inlineStr"/>
       <c r="H32" s="4" t="inlineStr"/>
-      <c r="I32" t="inlineStr"/>
       <c r="J32" s="3" t="inlineStr"/>
     </row>
     <row r="33">
@@ -1582,7 +1551,6 @@
       </c>
       <c r="G33" s="3" t="inlineStr"/>
       <c r="H33" s="4" t="inlineStr"/>
-      <c r="I33" t="inlineStr"/>
       <c r="J33" s="3" t="inlineStr"/>
     </row>
     <row r="34">
@@ -1616,7 +1584,6 @@
       </c>
       <c r="G34" s="3" t="inlineStr"/>
       <c r="H34" s="4" t="inlineStr"/>
-      <c r="I34" t="inlineStr"/>
       <c r="J34" s="3" t="inlineStr"/>
     </row>
     <row r="35">
@@ -1650,7 +1617,6 @@
       </c>
       <c r="G35" s="3" t="inlineStr"/>
       <c r="H35" s="4" t="inlineStr"/>
-      <c r="I35" t="inlineStr"/>
       <c r="J35" s="3" t="inlineStr"/>
     </row>
     <row r="36">
@@ -1684,7 +1650,6 @@
       </c>
       <c r="G36" s="3" t="inlineStr"/>
       <c r="H36" s="4" t="inlineStr"/>
-      <c r="I36" t="inlineStr"/>
       <c r="J36" s="3" t="inlineStr"/>
     </row>
     <row r="37">
@@ -1718,7 +1683,6 @@
       </c>
       <c r="G37" s="3" t="inlineStr"/>
       <c r="H37" s="4" t="inlineStr"/>
-      <c r="I37" t="inlineStr"/>
       <c r="J37" s="3" t="inlineStr"/>
     </row>
     <row r="38">
@@ -1752,7 +1716,6 @@
       </c>
       <c r="G38" s="3" t="inlineStr"/>
       <c r="H38" s="4" t="inlineStr"/>
-      <c r="I38" t="inlineStr"/>
       <c r="J38" s="3" t="inlineStr"/>
     </row>
     <row r="39">
@@ -1786,7 +1749,6 @@
       </c>
       <c r="G39" s="3" t="inlineStr"/>
       <c r="H39" s="4" t="inlineStr"/>
-      <c r="I39" t="inlineStr"/>
       <c r="J39" s="3" t="inlineStr"/>
     </row>
     <row r="40">
@@ -1820,7 +1782,6 @@
       </c>
       <c r="G40" s="3" t="inlineStr"/>
       <c r="H40" s="4" t="inlineStr"/>
-      <c r="I40" t="inlineStr"/>
       <c r="J40" s="3" t="inlineStr"/>
     </row>
     <row r="41">
@@ -1854,7 +1815,6 @@
       </c>
       <c r="G41" s="3" t="inlineStr"/>
       <c r="H41" s="4" t="inlineStr"/>
-      <c r="I41" t="inlineStr"/>
       <c r="J41" s="3" t="inlineStr"/>
     </row>
     <row r="42">
@@ -1888,7 +1848,6 @@
       </c>
       <c r="G42" s="3" t="inlineStr"/>
       <c r="H42" s="4" t="inlineStr"/>
-      <c r="I42" t="inlineStr"/>
       <c r="J42" s="3" t="inlineStr"/>
     </row>
     <row r="43">
@@ -1922,7 +1881,6 @@
       </c>
       <c r="G43" s="3" t="inlineStr"/>
       <c r="H43" s="4" t="inlineStr"/>
-      <c r="I43" t="inlineStr"/>
       <c r="J43" s="3" t="inlineStr"/>
     </row>
     <row r="44">
@@ -1956,7 +1914,6 @@
       </c>
       <c r="G44" s="3" t="inlineStr"/>
       <c r="H44" s="4" t="inlineStr"/>
-      <c r="I44" t="inlineStr"/>
       <c r="J44" s="3" t="inlineStr"/>
     </row>
     <row r="45">
@@ -1990,7 +1947,6 @@
       </c>
       <c r="G45" s="3" t="inlineStr"/>
       <c r="H45" s="4" t="inlineStr"/>
-      <c r="I45" t="inlineStr"/>
       <c r="J45" s="3" t="inlineStr"/>
     </row>
     <row r="46">
@@ -2024,7 +1980,6 @@
       </c>
       <c r="G46" s="3" t="inlineStr"/>
       <c r="H46" s="4" t="inlineStr"/>
-      <c r="I46" t="inlineStr"/>
       <c r="J46" s="3" t="inlineStr"/>
     </row>
     <row r="47">
@@ -2058,7 +2013,6 @@
       </c>
       <c r="G47" s="3" t="inlineStr"/>
       <c r="H47" s="4" t="inlineStr"/>
-      <c r="I47" t="inlineStr"/>
       <c r="J47" s="3" t="inlineStr"/>
     </row>
     <row r="48">
@@ -2092,7 +2046,6 @@
       </c>
       <c r="G48" s="3" t="inlineStr"/>
       <c r="H48" s="4" t="inlineStr"/>
-      <c r="I48" t="inlineStr"/>
       <c r="J48" s="3" t="inlineStr"/>
     </row>
     <row r="49">
@@ -2126,7 +2079,6 @@
       </c>
       <c r="G49" s="3" t="inlineStr"/>
       <c r="H49" s="4" t="inlineStr"/>
-      <c r="I49" t="inlineStr"/>
       <c r="J49" s="3" t="inlineStr"/>
     </row>
     <row r="50">
@@ -2160,7 +2112,6 @@
       </c>
       <c r="G50" s="3" t="inlineStr"/>
       <c r="H50" s="4" t="inlineStr"/>
-      <c r="I50" t="inlineStr"/>
       <c r="J50" s="3" t="inlineStr"/>
     </row>
     <row r="51">
@@ -2194,7 +2145,6 @@
       </c>
       <c r="G51" s="3" t="inlineStr"/>
       <c r="H51" s="4" t="inlineStr"/>
-      <c r="I51" t="inlineStr"/>
       <c r="J51" s="3" t="inlineStr"/>
     </row>
     <row r="52">
@@ -2228,7 +2178,6 @@
       </c>
       <c r="G52" s="3" t="inlineStr"/>
       <c r="H52" s="4" t="inlineStr"/>
-      <c r="I52" t="inlineStr"/>
       <c r="J52" s="3" t="inlineStr"/>
     </row>
     <row r="53">
@@ -2262,7 +2211,6 @@
       </c>
       <c r="G53" s="3" t="inlineStr"/>
       <c r="H53" s="4" t="inlineStr"/>
-      <c r="I53" t="inlineStr"/>
       <c r="J53" s="3" t="inlineStr"/>
     </row>
     <row r="54">
@@ -2296,7 +2244,6 @@
       </c>
       <c r="G54" s="3" t="inlineStr"/>
       <c r="H54" s="4" t="inlineStr"/>
-      <c r="I54" t="inlineStr"/>
       <c r="J54" s="3" t="inlineStr"/>
     </row>
     <row r="55">
@@ -2330,7 +2277,6 @@
       </c>
       <c r="G55" s="3" t="inlineStr"/>
       <c r="H55" s="4" t="inlineStr"/>
-      <c r="I55" t="inlineStr"/>
       <c r="J55" s="3" t="inlineStr"/>
     </row>
     <row r="56">
@@ -2364,7 +2310,6 @@
       </c>
       <c r="G56" s="3" t="inlineStr"/>
       <c r="H56" s="4" t="inlineStr"/>
-      <c r="I56" t="inlineStr"/>
       <c r="J56" s="3" t="inlineStr"/>
     </row>
     <row r="57">
@@ -2398,7 +2343,6 @@
       </c>
       <c r="G57" s="3" t="inlineStr"/>
       <c r="H57" s="4" t="inlineStr"/>
-      <c r="I57" t="inlineStr"/>
       <c r="J57" s="3" t="inlineStr"/>
     </row>
     <row r="58">
@@ -2432,7 +2376,6 @@
       </c>
       <c r="G58" s="3" t="inlineStr"/>
       <c r="H58" s="4" t="inlineStr"/>
-      <c r="I58" t="inlineStr"/>
       <c r="J58" s="3" t="inlineStr"/>
     </row>
     <row r="59">
@@ -2466,7 +2409,6 @@
       </c>
       <c r="G59" s="3" t="inlineStr"/>
       <c r="H59" s="4" t="inlineStr"/>
-      <c r="I59" t="inlineStr"/>
       <c r="J59" s="3" t="inlineStr"/>
     </row>
     <row r="60">
@@ -2500,7 +2442,6 @@
       </c>
       <c r="G60" s="3" t="inlineStr"/>
       <c r="H60" s="4" t="inlineStr"/>
-      <c r="I60" t="inlineStr"/>
       <c r="J60" s="3" t="inlineStr"/>
     </row>
     <row r="61">
@@ -2534,7 +2475,6 @@
       </c>
       <c r="G61" s="3" t="inlineStr"/>
       <c r="H61" s="4" t="inlineStr"/>
-      <c r="I61" t="inlineStr"/>
       <c r="J61" s="3" t="inlineStr"/>
     </row>
     <row r="62">
@@ -2568,7 +2508,6 @@
       </c>
       <c r="G62" s="3" t="inlineStr"/>
       <c r="H62" s="4" t="inlineStr"/>
-      <c r="I62" t="inlineStr"/>
       <c r="J62" s="3" t="inlineStr"/>
     </row>
     <row r="63">
@@ -2602,7 +2541,6 @@
       </c>
       <c r="G63" s="3" t="inlineStr"/>
       <c r="H63" s="4" t="inlineStr"/>
-      <c r="I63" t="inlineStr"/>
       <c r="J63" s="3" t="inlineStr"/>
     </row>
     <row r="64">
@@ -2636,7 +2574,6 @@
       </c>
       <c r="G64" s="3" t="inlineStr"/>
       <c r="H64" s="4" t="inlineStr"/>
-      <c r="I64" t="inlineStr"/>
       <c r="J64" s="3" t="inlineStr"/>
     </row>
     <row r="65">
@@ -2670,7 +2607,6 @@
       </c>
       <c r="G65" s="3" t="inlineStr"/>
       <c r="H65" s="4" t="inlineStr"/>
-      <c r="I65" t="inlineStr"/>
       <c r="J65" s="3" t="inlineStr"/>
     </row>
     <row r="66">
@@ -2704,7 +2640,6 @@
       </c>
       <c r="G66" s="3" t="inlineStr"/>
       <c r="H66" s="4" t="inlineStr"/>
-      <c r="I66" t="inlineStr"/>
       <c r="J66" s="3" t="inlineStr"/>
     </row>
     <row r="67">
@@ -2738,7 +2673,6 @@
       </c>
       <c r="G67" s="3" t="inlineStr"/>
       <c r="H67" s="4" t="inlineStr"/>
-      <c r="I67" t="inlineStr"/>
       <c r="J67" s="3" t="inlineStr"/>
     </row>
     <row r="68">
@@ -2772,7 +2706,6 @@
       </c>
       <c r="G68" s="3" t="inlineStr"/>
       <c r="H68" s="4" t="inlineStr"/>
-      <c r="I68" t="inlineStr"/>
       <c r="J68" s="3" t="inlineStr"/>
     </row>
     <row r="69">
@@ -2806,7 +2739,6 @@
       </c>
       <c r="G69" s="3" t="inlineStr"/>
       <c r="H69" s="4" t="inlineStr"/>
-      <c r="I69" t="inlineStr"/>
       <c r="J69" s="3" t="inlineStr"/>
     </row>
     <row r="70">
@@ -2840,7 +2772,6 @@
       </c>
       <c r="G70" s="3" t="inlineStr"/>
       <c r="H70" s="4" t="inlineStr"/>
-      <c r="I70" t="inlineStr"/>
       <c r="J70" s="3" t="inlineStr"/>
     </row>
     <row r="71">
@@ -2874,7 +2805,6 @@
       </c>
       <c r="G71" s="3" t="inlineStr"/>
       <c r="H71" s="4" t="inlineStr"/>
-      <c r="I71" t="inlineStr"/>
       <c r="J71" s="3" t="inlineStr"/>
     </row>
     <row r="72">
@@ -2908,7 +2838,6 @@
       </c>
       <c r="G72" s="3" t="inlineStr"/>
       <c r="H72" s="4" t="inlineStr"/>
-      <c r="I72" t="inlineStr"/>
       <c r="J72" s="3" t="inlineStr"/>
     </row>
     <row r="73">
@@ -2942,7 +2871,6 @@
       </c>
       <c r="G73" s="3" t="inlineStr"/>
       <c r="H73" s="4" t="inlineStr"/>
-      <c r="I73" t="inlineStr"/>
       <c r="J73" s="3" t="inlineStr"/>
     </row>
     <row r="74">
@@ -2976,7 +2904,6 @@
       </c>
       <c r="G74" s="3" t="inlineStr"/>
       <c r="H74" s="4" t="inlineStr"/>
-      <c r="I74" t="inlineStr"/>
       <c r="J74" s="3" t="inlineStr"/>
     </row>
     <row r="75">
@@ -3010,7 +2937,6 @@
       </c>
       <c r="G75" s="3" t="inlineStr"/>
       <c r="H75" s="4" t="inlineStr"/>
-      <c r="I75" t="inlineStr"/>
       <c r="J75" s="3" t="inlineStr"/>
     </row>
     <row r="76">
@@ -3044,7 +2970,6 @@
       </c>
       <c r="G76" s="3" t="inlineStr"/>
       <c r="H76" s="4" t="inlineStr"/>
-      <c r="I76" t="inlineStr"/>
       <c r="J76" s="3" t="inlineStr"/>
     </row>
     <row r="77">
@@ -3078,7 +3003,6 @@
       </c>
       <c r="G77" s="3" t="inlineStr"/>
       <c r="H77" s="4" t="inlineStr"/>
-      <c r="I77" t="inlineStr"/>
       <c r="J77" s="3" t="inlineStr"/>
     </row>
     <row r="78">
@@ -3112,7 +3036,6 @@
       </c>
       <c r="G78" s="3" t="inlineStr"/>
       <c r="H78" s="4" t="inlineStr"/>
-      <c r="I78" t="inlineStr"/>
       <c r="J78" s="3" t="inlineStr"/>
     </row>
     <row r="79">
@@ -3146,7 +3069,6 @@
       </c>
       <c r="G79" s="3" t="inlineStr"/>
       <c r="H79" s="4" t="inlineStr"/>
-      <c r="I79" t="inlineStr"/>
       <c r="J79" s="3" t="inlineStr"/>
     </row>
     <row r="80">
@@ -3180,7 +3102,6 @@
       </c>
       <c r="G80" s="3" t="inlineStr"/>
       <c r="H80" s="4" t="inlineStr"/>
-      <c r="I80" t="inlineStr"/>
       <c r="J80" s="3" t="inlineStr"/>
     </row>
     <row r="81">
@@ -3214,7 +3135,6 @@
       </c>
       <c r="G81" s="3" t="inlineStr"/>
       <c r="H81" s="4" t="inlineStr"/>
-      <c r="I81" t="inlineStr"/>
       <c r="J81" s="3" t="inlineStr"/>
     </row>
     <row r="82">
@@ -3248,7 +3168,6 @@
       </c>
       <c r="G82" s="3" t="inlineStr"/>
       <c r="H82" s="4" t="inlineStr"/>
-      <c r="I82" t="inlineStr"/>
       <c r="J82" s="3" t="inlineStr"/>
     </row>
     <row r="83">
@@ -3282,7 +3201,6 @@
       </c>
       <c r="G83" s="3" t="inlineStr"/>
       <c r="H83" s="4" t="inlineStr"/>
-      <c r="I83" t="inlineStr"/>
       <c r="J83" s="3" t="inlineStr"/>
     </row>
     <row r="84">
@@ -3316,7 +3234,6 @@
       </c>
       <c r="G84" s="3" t="inlineStr"/>
       <c r="H84" s="4" t="inlineStr"/>
-      <c r="I84" t="inlineStr"/>
       <c r="J84" s="3" t="inlineStr"/>
     </row>
     <row r="85">
@@ -3350,7 +3267,6 @@
       </c>
       <c r="G85" s="3" t="inlineStr"/>
       <c r="H85" s="4" t="inlineStr"/>
-      <c r="I85" t="inlineStr"/>
       <c r="J85" s="3" t="inlineStr"/>
     </row>
     <row r="86">
@@ -3384,7 +3300,6 @@
       </c>
       <c r="G86" s="3" t="inlineStr"/>
       <c r="H86" s="4" t="inlineStr"/>
-      <c r="I86" t="inlineStr"/>
       <c r="J86" s="3" t="inlineStr"/>
     </row>
     <row r="87">
@@ -3418,7 +3333,6 @@
       </c>
       <c r="G87" s="3" t="inlineStr"/>
       <c r="H87" s="4" t="inlineStr"/>
-      <c r="I87" t="inlineStr"/>
       <c r="J87" s="3" t="inlineStr"/>
     </row>
     <row r="88">
@@ -3452,7 +3366,6 @@
       </c>
       <c r="G88" s="3" t="inlineStr"/>
       <c r="H88" s="4" t="inlineStr"/>
-      <c r="I88" t="inlineStr"/>
       <c r="J88" s="3" t="inlineStr"/>
     </row>
     <row r="89">
@@ -3486,7 +3399,6 @@
       </c>
       <c r="G89" s="3" t="inlineStr"/>
       <c r="H89" s="4" t="inlineStr"/>
-      <c r="I89" t="inlineStr"/>
       <c r="J89" s="3" t="inlineStr"/>
     </row>
     <row r="90">
@@ -3520,7 +3432,6 @@
       </c>
       <c r="G90" s="3" t="inlineStr"/>
       <c r="H90" s="4" t="inlineStr"/>
-      <c r="I90" t="inlineStr"/>
       <c r="J90" s="3" t="inlineStr"/>
     </row>
     <row r="91">
@@ -3554,7 +3465,6 @@
       </c>
       <c r="G91" s="3" t="inlineStr"/>
       <c r="H91" s="4" t="inlineStr"/>
-      <c r="I91" t="inlineStr"/>
       <c r="J91" s="3" t="inlineStr"/>
     </row>
     <row r="92">
@@ -3588,7 +3498,6 @@
       </c>
       <c r="G92" s="3" t="inlineStr"/>
       <c r="H92" s="4" t="inlineStr"/>
-      <c r="I92" t="inlineStr"/>
       <c r="J92" s="3" t="inlineStr"/>
     </row>
     <row r="93">
@@ -3622,7 +3531,6 @@
       </c>
       <c r="G93" s="3" t="inlineStr"/>
       <c r="H93" s="4" t="inlineStr"/>
-      <c r="I93" t="inlineStr"/>
       <c r="J93" s="3" t="inlineStr"/>
     </row>
     <row r="94">
@@ -3656,7 +3564,6 @@
       </c>
       <c r="G94" s="3" t="inlineStr"/>
       <c r="H94" s="4" t="inlineStr"/>
-      <c r="I94" t="inlineStr"/>
       <c r="J94" s="3" t="inlineStr"/>
     </row>
     <row r="95">
@@ -3690,7 +3597,6 @@
       </c>
       <c r="G95" s="3" t="inlineStr"/>
       <c r="H95" s="4" t="inlineStr"/>
-      <c r="I95" t="inlineStr"/>
       <c r="J95" s="3" t="inlineStr"/>
     </row>
     <row r="96">
@@ -3724,7 +3630,6 @@
       </c>
       <c r="G96" s="3" t="inlineStr"/>
       <c r="H96" s="4" t="inlineStr"/>
-      <c r="I96" t="inlineStr"/>
       <c r="J96" s="3" t="inlineStr"/>
     </row>
     <row r="97">
@@ -3758,7 +3663,6 @@
       </c>
       <c r="G97" s="3" t="inlineStr"/>
       <c r="H97" s="4" t="inlineStr"/>
-      <c r="I97" t="inlineStr"/>
       <c r="J97" s="3" t="inlineStr"/>
     </row>
     <row r="98">
@@ -3792,7 +3696,6 @@
       </c>
       <c r="G98" s="3" t="inlineStr"/>
       <c r="H98" s="4" t="inlineStr"/>
-      <c r="I98" t="inlineStr"/>
       <c r="J98" s="3" t="inlineStr"/>
     </row>
     <row r="99">
@@ -3826,7 +3729,6 @@
       </c>
       <c r="G99" s="3" t="inlineStr"/>
       <c r="H99" s="4" t="inlineStr"/>
-      <c r="I99" t="inlineStr"/>
       <c r="J99" s="3" t="inlineStr"/>
     </row>
     <row r="100">
@@ -3860,7 +3762,6 @@
       </c>
       <c r="G100" s="3" t="inlineStr"/>
       <c r="H100" s="4" t="inlineStr"/>
-      <c r="I100" t="inlineStr"/>
       <c r="J100" s="3" t="inlineStr"/>
     </row>
     <row r="101">
@@ -3894,7 +3795,6 @@
       </c>
       <c r="G101" s="3" t="inlineStr"/>
       <c r="H101" s="4" t="inlineStr"/>
-      <c r="I101" t="inlineStr"/>
       <c r="J101" s="3" t="inlineStr"/>
     </row>
     <row r="102">
@@ -3928,7 +3828,6 @@
       </c>
       <c r="G102" s="3" t="inlineStr"/>
       <c r="H102" s="4" t="inlineStr"/>
-      <c r="I102" t="inlineStr"/>
       <c r="J102" s="3" t="inlineStr"/>
     </row>
     <row r="103">
@@ -3962,7 +3861,6 @@
       </c>
       <c r="G103" s="3" t="inlineStr"/>
       <c r="H103" s="4" t="inlineStr"/>
-      <c r="I103" t="inlineStr"/>
       <c r="J103" s="3" t="inlineStr"/>
     </row>
     <row r="104">
@@ -3996,7 +3894,6 @@
       </c>
       <c r="G104" s="3" t="inlineStr"/>
       <c r="H104" s="4" t="inlineStr"/>
-      <c r="I104" t="inlineStr"/>
       <c r="J104" s="3" t="inlineStr"/>
     </row>
     <row r="105">
@@ -4030,7 +3927,6 @@
       </c>
       <c r="G105" s="3" t="inlineStr"/>
       <c r="H105" s="4" t="inlineStr"/>
-      <c r="I105" t="inlineStr"/>
       <c r="J105" s="3" t="inlineStr"/>
     </row>
     <row r="106">
@@ -4064,7 +3960,6 @@
       </c>
       <c r="G106" s="3" t="inlineStr"/>
       <c r="H106" s="4" t="inlineStr"/>
-      <c r="I106" t="inlineStr"/>
       <c r="J106" s="3" t="inlineStr"/>
     </row>
     <row r="107">
@@ -4098,7 +3993,6 @@
       </c>
       <c r="G107" s="3" t="inlineStr"/>
       <c r="H107" s="4" t="inlineStr"/>
-      <c r="I107" t="inlineStr"/>
       <c r="J107" s="3" t="inlineStr"/>
     </row>
     <row r="108">
@@ -4132,7 +4026,6 @@
       </c>
       <c r="G108" s="3" t="inlineStr"/>
       <c r="H108" s="4" t="inlineStr"/>
-      <c r="I108" t="inlineStr"/>
       <c r="J108" s="3" t="inlineStr"/>
     </row>
     <row r="109">
@@ -4166,7 +4059,6 @@
       </c>
       <c r="G109" s="3" t="inlineStr"/>
       <c r="H109" s="4" t="inlineStr"/>
-      <c r="I109" t="inlineStr"/>
       <c r="J109" s="3" t="inlineStr"/>
     </row>
     <row r="110">
@@ -4200,7 +4092,6 @@
       </c>
       <c r="G110" s="3" t="inlineStr"/>
       <c r="H110" s="4" t="inlineStr"/>
-      <c r="I110" t="inlineStr"/>
       <c r="J110" s="3" t="inlineStr"/>
     </row>
     <row r="111">
@@ -4234,7 +4125,6 @@
       </c>
       <c r="G111" s="3" t="inlineStr"/>
       <c r="H111" s="4" t="inlineStr"/>
-      <c r="I111" t="inlineStr"/>
       <c r="J111" s="3" t="inlineStr"/>
     </row>
     <row r="112">
@@ -4268,7 +4158,6 @@
       </c>
       <c r="G112" s="3" t="inlineStr"/>
       <c r="H112" s="4" t="inlineStr"/>
-      <c r="I112" t="inlineStr"/>
       <c r="J112" s="3" t="inlineStr"/>
     </row>
     <row r="113">
@@ -4302,7 +4191,6 @@
       </c>
       <c r="G113" s="3" t="inlineStr"/>
       <c r="H113" s="4" t="inlineStr"/>
-      <c r="I113" t="inlineStr"/>
       <c r="J113" s="3" t="inlineStr"/>
     </row>
     <row r="114">
@@ -4336,7 +4224,6 @@
       </c>
       <c r="G114" s="3" t="inlineStr"/>
       <c r="H114" s="4" t="inlineStr"/>
-      <c r="I114" t="inlineStr"/>
       <c r="J114" s="3" t="inlineStr"/>
     </row>
     <row r="115">
@@ -4370,7 +4257,6 @@
       </c>
       <c r="G115" s="3" t="inlineStr"/>
       <c r="H115" s="4" t="inlineStr"/>
-      <c r="I115" t="inlineStr"/>
       <c r="J115" s="3" t="inlineStr"/>
     </row>
     <row r="116">
@@ -4404,7 +4290,6 @@
       </c>
       <c r="G116" s="3" t="inlineStr"/>
       <c r="H116" s="4" t="inlineStr"/>
-      <c r="I116" t="inlineStr"/>
       <c r="J116" s="3" t="inlineStr"/>
     </row>
     <row r="117">
@@ -4438,7 +4323,6 @@
       </c>
       <c r="G117" s="3" t="inlineStr"/>
       <c r="H117" s="4" t="inlineStr"/>
-      <c r="I117" t="inlineStr"/>
       <c r="J117" s="3" t="inlineStr"/>
     </row>
     <row r="118">
@@ -4472,7 +4356,6 @@
       </c>
       <c r="G118" s="3" t="inlineStr"/>
       <c r="H118" s="4" t="inlineStr"/>
-      <c r="I118" t="inlineStr"/>
       <c r="J118" s="3" t="inlineStr"/>
     </row>
     <row r="119">
@@ -4506,7 +4389,6 @@
       </c>
       <c r="G119" s="3" t="inlineStr"/>
       <c r="H119" s="4" t="inlineStr"/>
-      <c r="I119" t="inlineStr"/>
       <c r="J119" s="3" t="inlineStr"/>
     </row>
     <row r="120">
@@ -4540,7 +4422,6 @@
       </c>
       <c r="G120" s="3" t="inlineStr"/>
       <c r="H120" s="4" t="inlineStr"/>
-      <c r="I120" t="inlineStr"/>
       <c r="J120" s="3" t="inlineStr"/>
     </row>
     <row r="121">
@@ -4574,7 +4455,6 @@
       </c>
       <c r="G121" s="3" t="inlineStr"/>
       <c r="H121" s="4" t="inlineStr"/>
-      <c r="I121" t="inlineStr"/>
       <c r="J121" s="3" t="inlineStr"/>
     </row>
     <row r="122">
@@ -4608,7 +4488,6 @@
       </c>
       <c r="G122" s="3" t="inlineStr"/>
       <c r="H122" s="4" t="inlineStr"/>
-      <c r="I122" t="inlineStr"/>
       <c r="J122" s="3" t="inlineStr"/>
     </row>
     <row r="123">
@@ -4642,7 +4521,6 @@
       </c>
       <c r="G123" s="3" t="inlineStr"/>
       <c r="H123" s="4" t="inlineStr"/>
-      <c r="I123" t="inlineStr"/>
       <c r="J123" s="3" t="inlineStr"/>
     </row>
     <row r="124">
@@ -4676,7 +4554,6 @@
       </c>
       <c r="G124" s="3" t="inlineStr"/>
       <c r="H124" s="4" t="inlineStr"/>
-      <c r="I124" t="inlineStr"/>
       <c r="J124" s="3" t="inlineStr"/>
     </row>
     <row r="125">
@@ -4710,7 +4587,6 @@
       </c>
       <c r="G125" s="3" t="inlineStr"/>
       <c r="H125" s="4" t="inlineStr"/>
-      <c r="I125" t="inlineStr"/>
       <c r="J125" s="3" t="inlineStr"/>
     </row>
     <row r="126">
@@ -4744,7 +4620,6 @@
       </c>
       <c r="G126" s="3" t="inlineStr"/>
       <c r="H126" s="4" t="inlineStr"/>
-      <c r="I126" t="inlineStr"/>
       <c r="J126" s="3" t="inlineStr"/>
     </row>
     <row r="127">
@@ -4778,7 +4653,6 @@
       </c>
       <c r="G127" s="3" t="inlineStr"/>
       <c r="H127" s="4" t="inlineStr"/>
-      <c r="I127" t="inlineStr"/>
       <c r="J127" s="3" t="inlineStr"/>
     </row>
     <row r="128">
@@ -4812,7 +4686,6 @@
       </c>
       <c r="G128" s="3" t="inlineStr"/>
       <c r="H128" s="4" t="inlineStr"/>
-      <c r="I128" t="inlineStr"/>
       <c r="J128" s="3" t="inlineStr"/>
     </row>
     <row r="129">
@@ -4846,7 +4719,6 @@
       </c>
       <c r="G129" s="3" t="inlineStr"/>
       <c r="H129" s="4" t="inlineStr"/>
-      <c r="I129" t="inlineStr"/>
       <c r="J129" s="3" t="inlineStr"/>
     </row>
     <row r="130">
@@ -4880,7 +4752,6 @@
       </c>
       <c r="G130" s="3" t="inlineStr"/>
       <c r="H130" s="4" t="inlineStr"/>
-      <c r="I130" t="inlineStr"/>
       <c r="J130" s="3" t="inlineStr"/>
     </row>
     <row r="131">
@@ -4914,7 +4785,6 @@
       </c>
       <c r="G131" s="3" t="inlineStr"/>
       <c r="H131" s="4" t="inlineStr"/>
-      <c r="I131" t="inlineStr"/>
       <c r="J131" s="3" t="inlineStr"/>
     </row>
     <row r="132">
@@ -4948,7 +4818,6 @@
       </c>
       <c r="G132" s="3" t="inlineStr"/>
       <c r="H132" s="4" t="inlineStr"/>
-      <c r="I132" t="inlineStr"/>
       <c r="J132" s="3" t="inlineStr"/>
     </row>
     <row r="133">
@@ -4982,7 +4851,6 @@
       </c>
       <c r="G133" s="3" t="inlineStr"/>
       <c r="H133" s="4" t="inlineStr"/>
-      <c r="I133" t="inlineStr"/>
       <c r="J133" s="3" t="inlineStr"/>
     </row>
     <row r="134">
@@ -5016,7 +4884,6 @@
       </c>
       <c r="G134" s="3" t="inlineStr"/>
       <c r="H134" s="4" t="inlineStr"/>
-      <c r="I134" t="inlineStr"/>
       <c r="J134" s="3" t="inlineStr"/>
     </row>
     <row r="135">
@@ -5050,7 +4917,6 @@
       </c>
       <c r="G135" s="3" t="inlineStr"/>
       <c r="H135" s="4" t="inlineStr"/>
-      <c r="I135" t="inlineStr"/>
       <c r="J135" s="3" t="inlineStr"/>
     </row>
     <row r="136">
@@ -5084,7 +4950,6 @@
       </c>
       <c r="G136" s="3" t="inlineStr"/>
       <c r="H136" s="4" t="inlineStr"/>
-      <c r="I136" t="inlineStr"/>
       <c r="J136" s="3" t="inlineStr"/>
     </row>
     <row r="137">
@@ -5118,7 +4983,6 @@
       </c>
       <c r="G137" s="3" t="inlineStr"/>
       <c r="H137" s="4" t="inlineStr"/>
-      <c r="I137" t="inlineStr"/>
       <c r="J137" s="3" t="inlineStr"/>
     </row>
     <row r="138">
@@ -5152,7 +5016,6 @@
       </c>
       <c r="G138" s="3" t="inlineStr"/>
       <c r="H138" s="4" t="inlineStr"/>
-      <c r="I138" t="inlineStr"/>
       <c r="J138" s="3" t="inlineStr"/>
     </row>
     <row r="139">
@@ -5186,7 +5049,6 @@
       </c>
       <c r="G139" s="3" t="inlineStr"/>
       <c r="H139" s="4" t="inlineStr"/>
-      <c r="I139" t="inlineStr"/>
       <c r="J139" s="3" t="inlineStr"/>
     </row>
     <row r="140">
@@ -5220,7 +5082,6 @@
       </c>
       <c r="G140" s="3" t="inlineStr"/>
       <c r="H140" s="4" t="inlineStr"/>
-      <c r="I140" t="inlineStr"/>
       <c r="J140" s="3" t="inlineStr"/>
     </row>
     <row r="141">
@@ -5254,7 +5115,6 @@
       </c>
       <c r="G141" s="3" t="inlineStr"/>
       <c r="H141" s="4" t="inlineStr"/>
-      <c r="I141" t="inlineStr"/>
       <c r="J141" s="3" t="inlineStr"/>
     </row>
     <row r="142">
@@ -5288,7 +5148,6 @@
       </c>
       <c r="G142" s="3" t="inlineStr"/>
       <c r="H142" s="4" t="inlineStr"/>
-      <c r="I142" t="inlineStr"/>
       <c r="J142" s="3" t="inlineStr"/>
     </row>
     <row r="143">
@@ -5322,7 +5181,6 @@
       </c>
       <c r="G143" s="3" t="inlineStr"/>
       <c r="H143" s="4" t="inlineStr"/>
-      <c r="I143" t="inlineStr"/>
       <c r="J143" s="3" t="inlineStr"/>
     </row>
     <row r="144">
@@ -5356,7 +5214,6 @@
       </c>
       <c r="G144" s="3" t="inlineStr"/>
       <c r="H144" s="4" t="inlineStr"/>
-      <c r="I144" t="inlineStr"/>
       <c r="J144" s="3" t="inlineStr"/>
     </row>
     <row r="145">
@@ -5390,7 +5247,6 @@
       </c>
       <c r="G145" s="3" t="inlineStr"/>
       <c r="H145" s="4" t="inlineStr"/>
-      <c r="I145" t="inlineStr"/>
       <c r="J145" s="3" t="inlineStr"/>
     </row>
     <row r="146">
@@ -5424,7 +5280,6 @@
       </c>
       <c r="G146" s="3" t="inlineStr"/>
       <c r="H146" s="4" t="inlineStr"/>
-      <c r="I146" t="inlineStr"/>
       <c r="J146" s="3" t="inlineStr"/>
     </row>
     <row r="147">
@@ -5458,7 +5313,6 @@
       </c>
       <c r="G147" s="3" t="inlineStr"/>
       <c r="H147" s="4" t="inlineStr"/>
-      <c r="I147" t="inlineStr"/>
       <c r="J147" s="3" t="inlineStr"/>
     </row>
     <row r="148">
@@ -5492,7 +5346,6 @@
       </c>
       <c r="G148" s="3" t="inlineStr"/>
       <c r="H148" s="4" t="inlineStr"/>
-      <c r="I148" t="inlineStr"/>
       <c r="J148" s="3" t="inlineStr"/>
     </row>
     <row r="149">
@@ -5526,7 +5379,6 @@
       </c>
       <c r="G149" s="3" t="inlineStr"/>
       <c r="H149" s="4" t="inlineStr"/>
-      <c r="I149" t="inlineStr"/>
       <c r="J149" s="3" t="inlineStr"/>
     </row>
     <row r="150">
@@ -5560,7 +5412,6 @@
       </c>
       <c r="G150" s="3" t="inlineStr"/>
       <c r="H150" s="4" t="inlineStr"/>
-      <c r="I150" t="inlineStr"/>
       <c r="J150" s="3" t="inlineStr"/>
     </row>
     <row r="151">
@@ -5594,7 +5445,6 @@
       </c>
       <c r="G151" s="3" t="inlineStr"/>
       <c r="H151" s="4" t="inlineStr"/>
-      <c r="I151" t="inlineStr"/>
       <c r="J151" s="3" t="inlineStr"/>
     </row>
     <row r="152">
@@ -5628,7 +5478,6 @@
       </c>
       <c r="G152" s="3" t="inlineStr"/>
       <c r="H152" s="4" t="inlineStr"/>
-      <c r="I152" t="inlineStr"/>
       <c r="J152" s="3" t="inlineStr"/>
     </row>
     <row r="153">
@@ -5662,7 +5511,6 @@
       </c>
       <c r="G153" s="3" t="inlineStr"/>
       <c r="H153" s="4" t="inlineStr"/>
-      <c r="I153" t="inlineStr"/>
       <c r="J153" s="3" t="inlineStr"/>
     </row>
     <row r="154">
@@ -5696,7 +5544,6 @@
       </c>
       <c r="G154" s="3" t="inlineStr"/>
       <c r="H154" s="4" t="inlineStr"/>
-      <c r="I154" t="inlineStr"/>
       <c r="J154" s="3" t="inlineStr"/>
     </row>
     <row r="155">
@@ -5730,7 +5577,6 @@
       </c>
       <c r="G155" s="3" t="inlineStr"/>
       <c r="H155" s="4" t="inlineStr"/>
-      <c r="I155" t="inlineStr"/>
       <c r="J155" s="3" t="inlineStr"/>
     </row>
     <row r="156">
@@ -5764,7 +5610,6 @@
       </c>
       <c r="G156" s="3" t="inlineStr"/>
       <c r="H156" s="4" t="inlineStr"/>
-      <c r="I156" t="inlineStr"/>
       <c r="J156" s="3" t="inlineStr"/>
     </row>
     <row r="157">
@@ -5798,7 +5643,6 @@
       </c>
       <c r="G157" s="3" t="inlineStr"/>
       <c r="H157" s="4" t="inlineStr"/>
-      <c r="I157" t="inlineStr"/>
       <c r="J157" s="3" t="inlineStr"/>
     </row>
     <row r="158">
@@ -5832,7 +5676,6 @@
       </c>
       <c r="G158" s="3" t="inlineStr"/>
       <c r="H158" s="4" t="inlineStr"/>
-      <c r="I158" t="inlineStr"/>
       <c r="J158" s="3" t="inlineStr"/>
     </row>
     <row r="159">
@@ -5866,7 +5709,6 @@
       </c>
       <c r="G159" s="3" t="inlineStr"/>
       <c r="H159" s="4" t="inlineStr"/>
-      <c r="I159" t="inlineStr"/>
       <c r="J159" s="3" t="inlineStr"/>
     </row>
     <row r="160">
@@ -5900,7 +5742,6 @@
       </c>
       <c r="G160" s="3" t="inlineStr"/>
       <c r="H160" s="4" t="inlineStr"/>
-      <c r="I160" t="inlineStr"/>
       <c r="J160" s="3" t="inlineStr"/>
     </row>
     <row r="161">
@@ -5934,7 +5775,6 @@
       </c>
       <c r="G161" s="3" t="inlineStr"/>
       <c r="H161" s="4" t="inlineStr"/>
-      <c r="I161" t="inlineStr"/>
       <c r="J161" s="3" t="inlineStr"/>
     </row>
     <row r="162">
@@ -5968,7 +5808,6 @@
       </c>
       <c r="G162" s="3" t="inlineStr"/>
       <c r="H162" s="4" t="inlineStr"/>
-      <c r="I162" t="inlineStr"/>
       <c r="J162" s="3" t="inlineStr"/>
     </row>
     <row r="163">
@@ -6002,7 +5841,6 @@
       </c>
       <c r="G163" s="3" t="inlineStr"/>
       <c r="H163" s="4" t="inlineStr"/>
-      <c r="I163" t="inlineStr"/>
       <c r="J163" s="3" t="inlineStr"/>
     </row>
     <row r="164">
@@ -6036,7 +5874,6 @@
       </c>
       <c r="G164" s="3" t="inlineStr"/>
       <c r="H164" s="4" t="inlineStr"/>
-      <c r="I164" t="inlineStr"/>
       <c r="J164" s="3" t="inlineStr"/>
     </row>
     <row r="165">
@@ -6070,7 +5907,6 @@
       </c>
       <c r="G165" s="3" t="inlineStr"/>
       <c r="H165" s="4" t="inlineStr"/>
-      <c r="I165" t="inlineStr"/>
       <c r="J165" s="3" t="inlineStr"/>
     </row>
     <row r="166">
@@ -6104,7 +5940,6 @@
       </c>
       <c r="G166" s="3" t="inlineStr"/>
       <c r="H166" s="4" t="inlineStr"/>
-      <c r="I166" t="inlineStr"/>
       <c r="J166" s="3" t="inlineStr"/>
     </row>
     <row r="167">
@@ -6138,7 +5973,6 @@
       </c>
       <c r="G167" s="3" t="inlineStr"/>
       <c r="H167" s="4" t="inlineStr"/>
-      <c r="I167" t="inlineStr"/>
       <c r="J167" s="3" t="inlineStr"/>
     </row>
     <row r="168">
@@ -6172,7 +6006,6 @@
       </c>
       <c r="G168" s="3" t="inlineStr"/>
       <c r="H168" s="4" t="inlineStr"/>
-      <c r="I168" t="inlineStr"/>
       <c r="J168" s="3" t="inlineStr"/>
     </row>
     <row r="169">
@@ -6206,7 +6039,6 @@
       </c>
       <c r="G169" s="3" t="inlineStr"/>
       <c r="H169" s="4" t="inlineStr"/>
-      <c r="I169" t="inlineStr"/>
       <c r="J169" s="3" t="inlineStr"/>
     </row>
     <row r="170">
@@ -6240,7 +6072,6 @@
       </c>
       <c r="G170" s="3" t="inlineStr"/>
       <c r="H170" s="4" t="inlineStr"/>
-      <c r="I170" t="inlineStr"/>
       <c r="J170" s="3" t="inlineStr"/>
     </row>
     <row r="171">
@@ -6274,7 +6105,6 @@
       </c>
       <c r="G171" s="3" t="inlineStr"/>
       <c r="H171" s="4" t="inlineStr"/>
-      <c r="I171" t="inlineStr"/>
       <c r="J171" s="3" t="inlineStr"/>
     </row>
     <row r="172">
@@ -6308,7 +6138,6 @@
       </c>
       <c r="G172" s="3" t="inlineStr"/>
       <c r="H172" s="4" t="inlineStr"/>
-      <c r="I172" t="inlineStr"/>
       <c r="J172" s="3" t="inlineStr"/>
     </row>
     <row r="173">
@@ -6342,7 +6171,6 @@
       </c>
       <c r="G173" s="3" t="inlineStr"/>
       <c r="H173" s="4" t="inlineStr"/>
-      <c r="I173" t="inlineStr"/>
       <c r="J173" s="3" t="inlineStr"/>
     </row>
     <row r="174">
@@ -6376,7 +6204,6 @@
       </c>
       <c r="G174" s="3" t="inlineStr"/>
       <c r="H174" s="4" t="inlineStr"/>
-      <c r="I174" t="inlineStr"/>
       <c r="J174" s="3" t="inlineStr"/>
     </row>
     <row r="175">
@@ -6410,7 +6237,6 @@
       </c>
       <c r="G175" s="3" t="inlineStr"/>
       <c r="H175" s="4" t="inlineStr"/>
-      <c r="I175" t="inlineStr"/>
       <c r="J175" s="3" t="inlineStr"/>
     </row>
     <row r="176">
@@ -6444,7 +6270,6 @@
       </c>
       <c r="G176" s="3" t="inlineStr"/>
       <c r="H176" s="4" t="inlineStr"/>
-      <c r="I176" t="inlineStr"/>
       <c r="J176" s="3" t="inlineStr"/>
     </row>
     <row r="177">
@@ -6478,7 +6303,6 @@
       </c>
       <c r="G177" s="3" t="inlineStr"/>
       <c r="H177" s="4" t="inlineStr"/>
-      <c r="I177" t="inlineStr"/>
       <c r="J177" s="3" t="inlineStr"/>
     </row>
     <row r="178">
@@ -6512,7 +6336,6 @@
       </c>
       <c r="G178" s="3" t="inlineStr"/>
       <c r="H178" s="4" t="inlineStr"/>
-      <c r="I178" t="inlineStr"/>
       <c r="J178" s="3" t="inlineStr"/>
     </row>
     <row r="179">
@@ -6546,7 +6369,6 @@
       </c>
       <c r="G179" s="3" t="inlineStr"/>
       <c r="H179" s="4" t="inlineStr"/>
-      <c r="I179" t="inlineStr"/>
       <c r="J179" s="3" t="inlineStr"/>
     </row>
     <row r="180">
@@ -6580,7 +6402,6 @@
       </c>
       <c r="G180" s="3" t="inlineStr"/>
       <c r="H180" s="4" t="inlineStr"/>
-      <c r="I180" t="inlineStr"/>
       <c r="J180" s="3" t="inlineStr"/>
     </row>
     <row r="181">
@@ -6614,7 +6435,6 @@
       </c>
       <c r="G181" s="3" t="inlineStr"/>
       <c r="H181" s="4" t="inlineStr"/>
-      <c r="I181" t="inlineStr"/>
       <c r="J181" s="3" t="inlineStr"/>
     </row>
     <row r="182">
@@ -6648,7 +6468,6 @@
       </c>
       <c r="G182" s="3" t="inlineStr"/>
       <c r="H182" s="4" t="inlineStr"/>
-      <c r="I182" t="inlineStr"/>
       <c r="J182" s="3" t="inlineStr"/>
     </row>
     <row r="183">
@@ -6682,7 +6501,6 @@
       </c>
       <c r="G183" s="3" t="inlineStr"/>
       <c r="H183" s="4" t="inlineStr"/>
-      <c r="I183" t="inlineStr"/>
       <c r="J183" s="3" t="inlineStr"/>
     </row>
     <row r="184">
@@ -6716,7 +6534,6 @@
       </c>
       <c r="G184" s="3" t="inlineStr"/>
       <c r="H184" s="4" t="inlineStr"/>
-      <c r="I184" t="inlineStr"/>
       <c r="J184" s="3" t="inlineStr"/>
     </row>
     <row r="185">
@@ -6750,7 +6567,6 @@
       </c>
       <c r="G185" s="3" t="inlineStr"/>
       <c r="H185" s="4" t="inlineStr"/>
-      <c r="I185" t="inlineStr"/>
       <c r="J185" s="3" t="inlineStr"/>
     </row>
     <row r="186">
@@ -6784,7 +6600,6 @@
       </c>
       <c r="G186" s="3" t="inlineStr"/>
       <c r="H186" s="4" t="inlineStr"/>
-      <c r="I186" t="inlineStr"/>
       <c r="J186" s="3" t="inlineStr"/>
     </row>
     <row r="187">
@@ -6818,7 +6633,6 @@
       </c>
       <c r="G187" s="3" t="inlineStr"/>
       <c r="H187" s="4" t="inlineStr"/>
-      <c r="I187" t="inlineStr"/>
       <c r="J187" s="3" t="inlineStr"/>
     </row>
     <row r="188">
@@ -6852,7 +6666,6 @@
       </c>
       <c r="G188" s="3" t="inlineStr"/>
       <c r="H188" s="4" t="inlineStr"/>
-      <c r="I188" t="inlineStr"/>
       <c r="J188" s="3" t="inlineStr"/>
     </row>
     <row r="189">
@@ -6886,7 +6699,6 @@
       </c>
       <c r="G189" s="3" t="inlineStr"/>
       <c r="H189" s="4" t="inlineStr"/>
-      <c r="I189" t="inlineStr"/>
       <c r="J189" s="3" t="inlineStr"/>
     </row>
     <row r="190">
@@ -6920,7 +6732,6 @@
       </c>
       <c r="G190" s="3" t="inlineStr"/>
       <c r="H190" s="4" t="inlineStr"/>
-      <c r="I190" t="inlineStr"/>
       <c r="J190" s="3" t="inlineStr"/>
     </row>
     <row r="191">
@@ -6954,7 +6765,6 @@
       </c>
       <c r="G191" s="3" t="inlineStr"/>
       <c r="H191" s="4" t="inlineStr"/>
-      <c r="I191" t="inlineStr"/>
       <c r="J191" s="3" t="inlineStr"/>
     </row>
     <row r="192">
@@ -6988,7 +6798,6 @@
       </c>
       <c r="G192" s="3" t="inlineStr"/>
       <c r="H192" s="4" t="inlineStr"/>
-      <c r="I192" t="inlineStr"/>
       <c r="J192" s="3" t="inlineStr"/>
     </row>
     <row r="193">
@@ -7022,7 +6831,6 @@
       </c>
       <c r="G193" s="3" t="inlineStr"/>
       <c r="H193" s="4" t="inlineStr"/>
-      <c r="I193" t="inlineStr"/>
       <c r="J193" s="3" t="inlineStr"/>
     </row>
     <row r="194">
@@ -7056,7 +6864,6 @@
       </c>
       <c r="G194" s="3" t="inlineStr"/>
       <c r="H194" s="4" t="inlineStr"/>
-      <c r="I194" t="inlineStr"/>
       <c r="J194" s="3" t="inlineStr"/>
     </row>
     <row r="195">
@@ -7090,7 +6897,6 @@
       </c>
       <c r="G195" s="3" t="inlineStr"/>
       <c r="H195" s="4" t="inlineStr"/>
-      <c r="I195" t="inlineStr"/>
       <c r="J195" s="3" t="inlineStr"/>
     </row>
     <row r="196">
@@ -7124,7 +6930,6 @@
       </c>
       <c r="G196" s="3" t="inlineStr"/>
       <c r="H196" s="4" t="inlineStr"/>
-      <c r="I196" t="inlineStr"/>
       <c r="J196" s="3" t="inlineStr"/>
     </row>
     <row r="197">
@@ -7158,7 +6963,6 @@
       </c>
       <c r="G197" s="3" t="inlineStr"/>
       <c r="H197" s="4" t="inlineStr"/>
-      <c r="I197" t="inlineStr"/>
       <c r="J197" s="3" t="inlineStr"/>
     </row>
     <row r="198">
@@ -7192,7 +6996,6 @@
       </c>
       <c r="G198" s="3" t="inlineStr"/>
       <c r="H198" s="4" t="inlineStr"/>
-      <c r="I198" t="inlineStr"/>
       <c r="J198" s="3" t="inlineStr"/>
     </row>
     <row r="199">
@@ -7226,7 +7029,6 @@
       </c>
       <c r="G199" s="3" t="inlineStr"/>
       <c r="H199" s="4" t="inlineStr"/>
-      <c r="I199" t="inlineStr"/>
       <c r="J199" s="3" t="inlineStr"/>
     </row>
     <row r="200">
@@ -7260,7 +7062,6 @@
       </c>
       <c r="G200" s="3" t="inlineStr"/>
       <c r="H200" s="4" t="inlineStr"/>
-      <c r="I200" t="inlineStr"/>
       <c r="J200" s="3" t="inlineStr"/>
     </row>
     <row r="201">
@@ -7294,7 +7095,6 @@
       </c>
       <c r="G201" s="3" t="inlineStr"/>
       <c r="H201" s="4" t="inlineStr"/>
-      <c r="I201" t="inlineStr"/>
       <c r="J201" s="3" t="inlineStr"/>
     </row>
     <row r="202">
@@ -7328,7 +7128,6 @@
       </c>
       <c r="G202" s="3" t="inlineStr"/>
       <c r="H202" s="4" t="inlineStr"/>
-      <c r="I202" t="inlineStr"/>
       <c r="J202" s="3" t="inlineStr"/>
     </row>
     <row r="203">
@@ -7362,7 +7161,6 @@
       </c>
       <c r="G203" s="3" t="inlineStr"/>
       <c r="H203" s="4" t="inlineStr"/>
-      <c r="I203" t="inlineStr"/>
       <c r="J203" s="3" t="inlineStr"/>
     </row>
     <row r="204">
@@ -7396,7 +7194,6 @@
       </c>
       <c r="G204" s="3" t="inlineStr"/>
       <c r="H204" s="4" t="inlineStr"/>
-      <c r="I204" t="inlineStr"/>
       <c r="J204" s="3" t="inlineStr"/>
     </row>
     <row r="205">
@@ -7430,7 +7227,6 @@
       </c>
       <c r="G205" s="3" t="inlineStr"/>
       <c r="H205" s="4" t="inlineStr"/>
-      <c r="I205" t="inlineStr"/>
       <c r="J205" s="3" t="inlineStr"/>
     </row>
     <row r="206">
@@ -7464,7 +7260,6 @@
       </c>
       <c r="G206" s="3" t="inlineStr"/>
       <c r="H206" s="4" t="inlineStr"/>
-      <c r="I206" t="inlineStr"/>
       <c r="J206" s="3" t="inlineStr"/>
     </row>
     <row r="207">
@@ -7498,7 +7293,6 @@
       </c>
       <c r="G207" s="3" t="inlineStr"/>
       <c r="H207" s="4" t="inlineStr"/>
-      <c r="I207" t="inlineStr"/>
       <c r="J207" s="3" t="inlineStr"/>
     </row>
     <row r="208">
@@ -7532,7 +7326,6 @@
       </c>
       <c r="G208" s="3" t="inlineStr"/>
       <c r="H208" s="4" t="inlineStr"/>
-      <c r="I208" t="inlineStr"/>
       <c r="J208" s="3" t="inlineStr"/>
     </row>
     <row r="209">
@@ -7566,7 +7359,6 @@
       </c>
       <c r="G209" s="3" t="inlineStr"/>
       <c r="H209" s="4" t="inlineStr"/>
-      <c r="I209" t="inlineStr"/>
       <c r="J209" s="3" t="inlineStr"/>
     </row>
     <row r="210">
@@ -7600,7 +7392,6 @@
       </c>
       <c r="G210" s="3" t="inlineStr"/>
       <c r="H210" s="4" t="inlineStr"/>
-      <c r="I210" t="inlineStr"/>
       <c r="J210" s="3" t="inlineStr"/>
     </row>
     <row r="211">
@@ -7634,7 +7425,6 @@
       </c>
       <c r="G211" s="3" t="inlineStr"/>
       <c r="H211" s="4" t="inlineStr"/>
-      <c r="I211" t="inlineStr"/>
       <c r="J211" s="3" t="inlineStr"/>
     </row>
     <row r="212">
@@ -7668,7 +7458,6 @@
       </c>
       <c r="G212" s="3" t="inlineStr"/>
       <c r="H212" s="4" t="inlineStr"/>
-      <c r="I212" t="inlineStr"/>
       <c r="J212" s="3" t="inlineStr"/>
     </row>
     <row r="213">
@@ -7702,7 +7491,6 @@
       </c>
       <c r="G213" s="3" t="inlineStr"/>
       <c r="H213" s="4" t="inlineStr"/>
-      <c r="I213" t="inlineStr"/>
       <c r="J213" s="3" t="inlineStr"/>
     </row>
     <row r="214">
@@ -7736,7 +7524,6 @@
       </c>
       <c r="G214" s="3" t="inlineStr"/>
       <c r="H214" s="4" t="inlineStr"/>
-      <c r="I214" t="inlineStr"/>
       <c r="J214" s="3" t="inlineStr"/>
     </row>
     <row r="215">
@@ -7770,7 +7557,6 @@
       </c>
       <c r="G215" s="3" t="inlineStr"/>
       <c r="H215" s="4" t="inlineStr"/>
-      <c r="I215" t="inlineStr"/>
       <c r="J215" s="3" t="inlineStr"/>
     </row>
     <row r="216">
@@ -7804,7 +7590,6 @@
       </c>
       <c r="G216" s="3" t="inlineStr"/>
       <c r="H216" s="4" t="inlineStr"/>
-      <c r="I216" t="inlineStr"/>
       <c r="J216" s="3" t="inlineStr"/>
     </row>
     <row r="217">
@@ -7838,7 +7623,6 @@
       </c>
       <c r="G217" s="3" t="inlineStr"/>
       <c r="H217" s="4" t="inlineStr"/>
-      <c r="I217" t="inlineStr"/>
       <c r="J217" s="3" t="inlineStr"/>
     </row>
     <row r="218">
@@ -7872,7 +7656,6 @@
       </c>
       <c r="G218" s="3" t="inlineStr"/>
       <c r="H218" s="4" t="inlineStr"/>
-      <c r="I218" t="inlineStr"/>
       <c r="J218" s="3" t="inlineStr"/>
     </row>
     <row r="219">
@@ -7906,7 +7689,6 @@
       </c>
       <c r="G219" s="3" t="inlineStr"/>
       <c r="H219" s="4" t="inlineStr"/>
-      <c r="I219" t="inlineStr"/>
       <c r="J219" s="3" t="inlineStr"/>
     </row>
     <row r="220">
@@ -7940,7 +7722,6 @@
       </c>
       <c r="G220" s="3" t="inlineStr"/>
       <c r="H220" s="4" t="inlineStr"/>
-      <c r="I220" t="inlineStr"/>
       <c r="J220" s="3" t="inlineStr"/>
     </row>
     <row r="221">
@@ -7974,7 +7755,6 @@
       </c>
       <c r="G221" s="3" t="inlineStr"/>
       <c r="H221" s="4" t="inlineStr"/>
-      <c r="I221" t="inlineStr"/>
       <c r="J221" s="3" t="inlineStr"/>
     </row>
     <row r="222">
@@ -8008,7 +7788,6 @@
       </c>
       <c r="G222" s="3" t="inlineStr"/>
       <c r="H222" s="4" t="inlineStr"/>
-      <c r="I222" t="inlineStr"/>
       <c r="J222" s="3" t="inlineStr"/>
     </row>
     <row r="223">
@@ -8042,7 +7821,6 @@
       </c>
       <c r="G223" s="3" t="inlineStr"/>
       <c r="H223" s="4" t="inlineStr"/>
-      <c r="I223" t="inlineStr"/>
       <c r="J223" s="3" t="inlineStr"/>
     </row>
     <row r="224">
@@ -8076,7 +7854,6 @@
       </c>
       <c r="G224" s="3" t="inlineStr"/>
       <c r="H224" s="4" t="inlineStr"/>
-      <c r="I224" t="inlineStr"/>
       <c r="J224" s="3" t="inlineStr"/>
     </row>
     <row r="225">
@@ -8110,7 +7887,6 @@
       </c>
       <c r="G225" s="3" t="inlineStr"/>
       <c r="H225" s="4" t="inlineStr"/>
-      <c r="I225" t="inlineStr"/>
       <c r="J225" s="3" t="inlineStr"/>
     </row>
     <row r="226">
@@ -8144,7 +7920,6 @@
       </c>
       <c r="G226" s="3" t="inlineStr"/>
       <c r="H226" s="4" t="inlineStr"/>
-      <c r="I226" t="inlineStr"/>
       <c r="J226" s="3" t="inlineStr"/>
     </row>
     <row r="227">
@@ -8178,7 +7953,6 @@
       </c>
       <c r="G227" s="3" t="inlineStr"/>
       <c r="H227" s="4" t="inlineStr"/>
-      <c r="I227" t="inlineStr"/>
       <c r="J227" s="3" t="inlineStr"/>
     </row>
     <row r="228">
@@ -8212,7 +7986,6 @@
       </c>
       <c r="G228" s="3" t="inlineStr"/>
       <c r="H228" s="4" t="inlineStr"/>
-      <c r="I228" t="inlineStr"/>
       <c r="J228" s="3" t="inlineStr"/>
     </row>
     <row r="229">
@@ -8246,7 +8019,6 @@
       </c>
       <c r="G229" s="3" t="inlineStr"/>
       <c r="H229" s="4" t="inlineStr"/>
-      <c r="I229" t="inlineStr"/>
       <c r="J229" s="3" t="inlineStr"/>
     </row>
     <row r="230">
@@ -8280,7 +8052,6 @@
       </c>
       <c r="G230" s="3" t="inlineStr"/>
       <c r="H230" s="4" t="inlineStr"/>
-      <c r="I230" t="inlineStr"/>
       <c r="J230" s="3" t="inlineStr"/>
     </row>
     <row r="231">
@@ -8314,7 +8085,6 @@
       </c>
       <c r="G231" s="3" t="inlineStr"/>
       <c r="H231" s="4" t="inlineStr"/>
-      <c r="I231" t="inlineStr"/>
       <c r="J231" s="3" t="inlineStr"/>
     </row>
     <row r="232">
@@ -8348,7 +8118,6 @@
       </c>
       <c r="G232" s="3" t="inlineStr"/>
       <c r="H232" s="4" t="inlineStr"/>
-      <c r="I232" t="inlineStr"/>
       <c r="J232" s="3" t="inlineStr"/>
     </row>
     <row r="233">
@@ -8382,7 +8151,6 @@
       </c>
       <c r="G233" s="3" t="inlineStr"/>
       <c r="H233" s="4" t="inlineStr"/>
-      <c r="I233" t="inlineStr"/>
       <c r="J233" s="3" t="inlineStr"/>
     </row>
     <row r="234">
@@ -8416,7 +8184,6 @@
       </c>
       <c r="G234" s="3" t="inlineStr"/>
       <c r="H234" s="4" t="inlineStr"/>
-      <c r="I234" t="inlineStr"/>
       <c r="J234" s="3" t="inlineStr"/>
     </row>
     <row r="235">
@@ -8450,7 +8217,6 @@
       </c>
       <c r="G235" s="3" t="inlineStr"/>
       <c r="H235" s="4" t="inlineStr"/>
-      <c r="I235" t="inlineStr"/>
       <c r="J235" s="3" t="inlineStr"/>
     </row>
     <row r="236">
@@ -8484,7 +8250,6 @@
       </c>
       <c r="G236" s="3" t="inlineStr"/>
       <c r="H236" s="4" t="inlineStr"/>
-      <c r="I236" t="inlineStr"/>
       <c r="J236" s="3" t="inlineStr"/>
     </row>
     <row r="237">
@@ -8518,7 +8283,6 @@
       </c>
       <c r="G237" s="3" t="inlineStr"/>
       <c r="H237" s="4" t="inlineStr"/>
-      <c r="I237" t="inlineStr"/>
       <c r="J237" s="3" t="inlineStr"/>
     </row>
     <row r="238">
@@ -8552,7 +8316,6 @@
       </c>
       <c r="G238" s="3" t="inlineStr"/>
       <c r="H238" s="4" t="inlineStr"/>
-      <c r="I238" t="inlineStr"/>
       <c r="J238" s="3" t="inlineStr"/>
     </row>
     <row r="239">
@@ -8586,7 +8349,6 @@
       </c>
       <c r="G239" s="3" t="inlineStr"/>
       <c r="H239" s="4" t="inlineStr"/>
-      <c r="I239" t="inlineStr"/>
       <c r="J239" s="3" t="inlineStr"/>
     </row>
     <row r="240">
@@ -8620,7 +8382,6 @@
       </c>
       <c r="G240" s="3" t="inlineStr"/>
       <c r="H240" s="4" t="inlineStr"/>
-      <c r="I240" t="inlineStr"/>
       <c r="J240" s="3" t="inlineStr"/>
     </row>
     <row r="241">
@@ -8654,7 +8415,6 @@
       </c>
       <c r="G241" s="3" t="inlineStr"/>
       <c r="H241" s="4" t="inlineStr"/>
-      <c r="I241" t="inlineStr"/>
       <c r="J241" s="3" t="inlineStr"/>
     </row>
     <row r="242">
@@ -8688,7 +8448,6 @@
       </c>
       <c r="G242" s="3" t="inlineStr"/>
       <c r="H242" s="4" t="inlineStr"/>
-      <c r="I242" t="inlineStr"/>
       <c r="J242" s="3" t="inlineStr"/>
     </row>
     <row r="243">
@@ -8722,7 +8481,6 @@
       </c>
       <c r="G243" s="3" t="inlineStr"/>
       <c r="H243" s="4" t="inlineStr"/>
-      <c r="I243" t="inlineStr"/>
       <c r="J243" s="3" t="inlineStr"/>
     </row>
     <row r="244">
@@ -8756,7 +8514,6 @@
       </c>
       <c r="G244" s="3" t="inlineStr"/>
       <c r="H244" s="4" t="inlineStr"/>
-      <c r="I244" t="inlineStr"/>
       <c r="J244" s="3" t="inlineStr"/>
     </row>
     <row r="245">
@@ -8790,7 +8547,6 @@
       </c>
       <c r="G245" s="3" t="inlineStr"/>
       <c r="H245" s="4" t="inlineStr"/>
-      <c r="I245" t="inlineStr"/>
       <c r="J245" s="3" t="inlineStr"/>
     </row>
     <row r="246">
@@ -8824,7 +8580,6 @@
       </c>
       <c r="G246" s="3" t="inlineStr"/>
       <c r="H246" s="4" t="inlineStr"/>
-      <c r="I246" t="inlineStr"/>
       <c r="J246" s="3" t="inlineStr"/>
     </row>
     <row r="247">
@@ -8858,7 +8613,6 @@
       </c>
       <c r="G247" s="3" t="inlineStr"/>
       <c r="H247" s="4" t="inlineStr"/>
-      <c r="I247" t="inlineStr"/>
       <c r="J247" s="3" t="inlineStr"/>
     </row>
     <row r="248">
@@ -8892,7 +8646,6 @@
       </c>
       <c r="G248" s="3" t="inlineStr"/>
       <c r="H248" s="4" t="inlineStr"/>
-      <c r="I248" t="inlineStr"/>
       <c r="J248" s="3" t="inlineStr"/>
     </row>
     <row r="249">
@@ -8926,7 +8679,6 @@
       </c>
       <c r="G249" s="3" t="inlineStr"/>
       <c r="H249" s="4" t="inlineStr"/>
-      <c r="I249" t="inlineStr"/>
       <c r="J249" s="3" t="inlineStr"/>
     </row>
     <row r="250">
@@ -8960,7 +8712,6 @@
       </c>
       <c r="G250" s="3" t="inlineStr"/>
       <c r="H250" s="4" t="inlineStr"/>
-      <c r="I250" t="inlineStr"/>
       <c r="J250" s="3" t="inlineStr"/>
     </row>
     <row r="251">
@@ -8994,7 +8745,6 @@
       </c>
       <c r="G251" s="3" t="inlineStr"/>
       <c r="H251" s="4" t="inlineStr"/>
-      <c r="I251" t="inlineStr"/>
       <c r="J251" s="3" t="inlineStr"/>
     </row>
     <row r="252">
@@ -9028,7 +8778,6 @@
       </c>
       <c r="G252" s="3" t="inlineStr"/>
       <c r="H252" s="4" t="inlineStr"/>
-      <c r="I252" t="inlineStr"/>
       <c r="J252" s="3" t="inlineStr"/>
     </row>
     <row r="253">
@@ -9062,7 +8811,6 @@
       </c>
       <c r="G253" s="3" t="inlineStr"/>
       <c r="H253" s="4" t="inlineStr"/>
-      <c r="I253" t="inlineStr"/>
       <c r="J253" s="3" t="inlineStr"/>
     </row>
     <row r="254">
@@ -9096,7 +8844,6 @@
       </c>
       <c r="G254" s="3" t="inlineStr"/>
       <c r="H254" s="4" t="inlineStr"/>
-      <c r="I254" t="inlineStr"/>
       <c r="J254" s="3" t="inlineStr"/>
     </row>
     <row r="255">
@@ -9130,7 +8877,6 @@
       </c>
       <c r="G255" s="3" t="inlineStr"/>
       <c r="H255" s="4" t="inlineStr"/>
-      <c r="I255" t="inlineStr"/>
       <c r="J255" s="3" t="inlineStr"/>
     </row>
     <row r="256">
@@ -9164,7 +8910,6 @@
       </c>
       <c r="G256" s="3" t="inlineStr"/>
       <c r="H256" s="4" t="inlineStr"/>
-      <c r="I256" t="inlineStr"/>
       <c r="J256" s="3" t="inlineStr"/>
     </row>
     <row r="257">
@@ -9198,7 +8943,6 @@
       </c>
       <c r="G257" s="3" t="inlineStr"/>
       <c r="H257" s="4" t="inlineStr"/>
-      <c r="I257" t="inlineStr"/>
       <c r="J257" s="3" t="inlineStr"/>
     </row>
     <row r="258">
@@ -9232,7 +8976,6 @@
       </c>
       <c r="G258" s="3" t="inlineStr"/>
       <c r="H258" s="4" t="inlineStr"/>
-      <c r="I258" t="inlineStr"/>
       <c r="J258" s="3" t="inlineStr"/>
     </row>
     <row r="259">
@@ -9266,7 +9009,6 @@
       </c>
       <c r="G259" s="3" t="inlineStr"/>
       <c r="H259" s="4" t="inlineStr"/>
-      <c r="I259" t="inlineStr"/>
       <c r="J259" s="3" t="inlineStr"/>
     </row>
     <row r="260">
@@ -9300,7 +9042,6 @@
       </c>
       <c r="G260" s="3" t="inlineStr"/>
       <c r="H260" s="4" t="inlineStr"/>
-      <c r="I260" t="inlineStr"/>
       <c r="J260" s="3" t="inlineStr"/>
     </row>
     <row r="261">
@@ -9334,7 +9075,6 @@
       </c>
       <c r="G261" s="3" t="inlineStr"/>
       <c r="H261" s="4" t="inlineStr"/>
-      <c r="I261" t="inlineStr"/>
       <c r="J261" s="3" t="inlineStr"/>
     </row>
     <row r="262">
@@ -9368,7 +9108,6 @@
       </c>
       <c r="G262" s="3" t="inlineStr"/>
       <c r="H262" s="4" t="inlineStr"/>
-      <c r="I262" t="inlineStr"/>
       <c r="J262" s="3" t="inlineStr"/>
     </row>
     <row r="263">
@@ -9402,7 +9141,6 @@
       </c>
       <c r="G263" s="3" t="inlineStr"/>
       <c r="H263" s="4" t="inlineStr"/>
-      <c r="I263" t="inlineStr"/>
       <c r="J263" s="3" t="inlineStr"/>
     </row>
     <row r="264">
@@ -9436,7 +9174,6 @@
       </c>
       <c r="G264" s="3" t="inlineStr"/>
       <c r="H264" s="4" t="inlineStr"/>
-      <c r="I264" t="inlineStr"/>
       <c r="J264" s="3" t="inlineStr"/>
     </row>
     <row r="265">
@@ -9470,7 +9207,6 @@
       </c>
       <c r="G265" s="3" t="inlineStr"/>
       <c r="H265" s="4" t="inlineStr"/>
-      <c r="I265" t="inlineStr"/>
       <c r="J265" s="3" t="inlineStr"/>
     </row>
     <row r="266">
@@ -9504,7 +9240,6 @@
       </c>
       <c r="G266" s="3" t="inlineStr"/>
       <c r="H266" s="4" t="inlineStr"/>
-      <c r="I266" t="inlineStr"/>
       <c r="J266" s="3" t="inlineStr"/>
     </row>
     <row r="267">
@@ -9538,7 +9273,6 @@
       </c>
       <c r="G267" s="3" t="inlineStr"/>
       <c r="H267" s="4" t="inlineStr"/>
-      <c r="I267" t="inlineStr"/>
       <c r="J267" s="3" t="inlineStr"/>
     </row>
     <row r="268">
@@ -9572,7 +9306,6 @@
       </c>
       <c r="G268" s="3" t="inlineStr"/>
       <c r="H268" s="4" t="inlineStr"/>
-      <c r="I268" t="inlineStr"/>
       <c r="J268" s="3" t="inlineStr"/>
     </row>
     <row r="269">
@@ -9606,7 +9339,6 @@
       </c>
       <c r="G269" s="3" t="inlineStr"/>
       <c r="H269" s="4" t="inlineStr"/>
-      <c r="I269" t="inlineStr"/>
       <c r="J269" s="3" t="inlineStr"/>
     </row>
     <row r="270">
@@ -9640,7 +9372,6 @@
       </c>
       <c r="G270" s="3" t="inlineStr"/>
       <c r="H270" s="4" t="inlineStr"/>
-      <c r="I270" t="inlineStr"/>
       <c r="J270" s="3" t="inlineStr"/>
     </row>
     <row r="271">
@@ -9674,7 +9405,6 @@
       </c>
       <c r="G271" s="3" t="inlineStr"/>
       <c r="H271" s="4" t="inlineStr"/>
-      <c r="I271" t="inlineStr"/>
       <c r="J271" s="3" t="inlineStr"/>
     </row>
     <row r="272">
@@ -9708,7 +9438,6 @@
       </c>
       <c r="G272" s="3" t="inlineStr"/>
       <c r="H272" s="4" t="inlineStr"/>
-      <c r="I272" t="inlineStr"/>
       <c r="J272" s="3" t="inlineStr"/>
     </row>
     <row r="273">
@@ -9742,7 +9471,6 @@
       </c>
       <c r="G273" s="3" t="inlineStr"/>
       <c r="H273" s="4" t="inlineStr"/>
-      <c r="I273" t="inlineStr"/>
       <c r="J273" s="3" t="inlineStr"/>
     </row>
     <row r="274">
@@ -9776,7 +9504,6 @@
       </c>
       <c r="G274" s="3" t="inlineStr"/>
       <c r="H274" s="4" t="inlineStr"/>
-      <c r="I274" t="inlineStr"/>
       <c r="J274" s="3" t="inlineStr"/>
     </row>
     <row r="275">
@@ -9810,7 +9537,6 @@
       </c>
       <c r="G275" s="3" t="inlineStr"/>
       <c r="H275" s="4" t="inlineStr"/>
-      <c r="I275" t="inlineStr"/>
       <c r="J275" s="3" t="inlineStr"/>
     </row>
     <row r="276">
@@ -9844,7 +9570,6 @@
       </c>
       <c r="G276" s="3" t="inlineStr"/>
       <c r="H276" s="4" t="inlineStr"/>
-      <c r="I276" t="inlineStr"/>
       <c r="J276" s="3" t="inlineStr"/>
     </row>
     <row r="277">
@@ -9878,7 +9603,6 @@
       </c>
       <c r="G277" s="3" t="inlineStr"/>
       <c r="H277" s="4" t="inlineStr"/>
-      <c r="I277" t="inlineStr"/>
       <c r="J277" s="3" t="inlineStr"/>
     </row>
     <row r="278">
@@ -9912,7 +9636,6 @@
       </c>
       <c r="G278" s="3" t="inlineStr"/>
       <c r="H278" s="4" t="inlineStr"/>
-      <c r="I278" t="inlineStr"/>
       <c r="J278" s="3" t="inlineStr"/>
     </row>
     <row r="279">
@@ -9946,7 +9669,6 @@
       </c>
       <c r="G279" s="3" t="inlineStr"/>
       <c r="H279" s="4" t="inlineStr"/>
-      <c r="I279" t="inlineStr"/>
       <c r="J279" s="3" t="inlineStr"/>
     </row>
     <row r="280">
@@ -9980,7 +9702,6 @@
       </c>
       <c r="G280" s="3" t="inlineStr"/>
       <c r="H280" s="4" t="inlineStr"/>
-      <c r="I280" t="inlineStr"/>
       <c r="J280" s="3" t="inlineStr"/>
     </row>
     <row r="281">
@@ -10014,7 +9735,6 @@
       </c>
       <c r="G281" s="3" t="inlineStr"/>
       <c r="H281" s="4" t="inlineStr"/>
-      <c r="I281" t="inlineStr"/>
       <c r="J281" s="3" t="inlineStr"/>
     </row>
     <row r="282">
@@ -10048,7 +9768,6 @@
       </c>
       <c r="G282" s="3" t="inlineStr"/>
       <c r="H282" s="4" t="inlineStr"/>
-      <c r="I282" t="inlineStr"/>
       <c r="J282" s="3" t="inlineStr"/>
     </row>
     <row r="283">
@@ -10082,7 +9801,6 @@
       </c>
       <c r="G283" s="3" t="inlineStr"/>
       <c r="H283" s="4" t="inlineStr"/>
-      <c r="I283" t="inlineStr"/>
       <c r="J283" s="3" t="inlineStr"/>
     </row>
     <row r="284">
@@ -10116,7 +9834,6 @@
       </c>
       <c r="G284" s="3" t="inlineStr"/>
       <c r="H284" s="4" t="inlineStr"/>
-      <c r="I284" t="inlineStr"/>
       <c r="J284" s="3" t="inlineStr"/>
     </row>
     <row r="285">
@@ -10150,7 +9867,6 @@
       </c>
       <c r="G285" s="3" t="inlineStr"/>
       <c r="H285" s="4" t="inlineStr"/>
-      <c r="I285" t="inlineStr"/>
       <c r="J285" s="3" t="inlineStr"/>
     </row>
     <row r="286">
@@ -10184,7 +9900,6 @@
       </c>
       <c r="G286" s="3" t="inlineStr"/>
       <c r="H286" s="4" t="inlineStr"/>
-      <c r="I286" t="inlineStr"/>
       <c r="J286" s="3" t="inlineStr"/>
     </row>
     <row r="287">
@@ -10218,7 +9933,6 @@
       </c>
       <c r="G287" s="3" t="inlineStr"/>
       <c r="H287" s="4" t="inlineStr"/>
-      <c r="I287" t="inlineStr"/>
       <c r="J287" s="3" t="inlineStr"/>
     </row>
     <row r="288">
@@ -10252,7 +9966,6 @@
       </c>
       <c r="G288" s="3" t="inlineStr"/>
       <c r="H288" s="4" t="inlineStr"/>
-      <c r="I288" t="inlineStr"/>
       <c r="J288" s="3" t="inlineStr"/>
     </row>
     <row r="289">
@@ -10286,7 +9999,6 @@
       </c>
       <c r="G289" s="3" t="inlineStr"/>
       <c r="H289" s="4" t="inlineStr"/>
-      <c r="I289" t="inlineStr"/>
       <c r="J289" s="3" t="inlineStr"/>
     </row>
     <row r="290">
@@ -10320,7 +10032,6 @@
       </c>
       <c r="G290" s="3" t="inlineStr"/>
       <c r="H290" s="4" t="inlineStr"/>
-      <c r="I290" t="inlineStr"/>
       <c r="J290" s="3" t="inlineStr"/>
     </row>
     <row r="291">
@@ -10354,7 +10065,6 @@
       </c>
       <c r="G291" s="3" t="inlineStr"/>
       <c r="H291" s="4" t="inlineStr"/>
-      <c r="I291" t="inlineStr"/>
       <c r="J291" s="3" t="inlineStr"/>
     </row>
     <row r="292">
@@ -10388,7 +10098,6 @@
       </c>
       <c r="G292" s="3" t="inlineStr"/>
       <c r="H292" s="4" t="inlineStr"/>
-      <c r="I292" t="inlineStr"/>
       <c r="J292" s="3" t="inlineStr"/>
     </row>
     <row r="293">
@@ -10422,7 +10131,6 @@
       </c>
       <c r="G293" s="3" t="inlineStr"/>
       <c r="H293" s="4" t="inlineStr"/>
-      <c r="I293" t="inlineStr"/>
       <c r="J293" s="3" t="inlineStr"/>
     </row>
     <row r="294">
@@ -10456,7 +10164,6 @@
       </c>
       <c r="G294" s="3" t="inlineStr"/>
       <c r="H294" s="4" t="inlineStr"/>
-      <c r="I294" t="inlineStr"/>
       <c r="J294" s="3" t="inlineStr"/>
     </row>
     <row r="295">
@@ -10490,7 +10197,6 @@
       </c>
       <c r="G295" s="3" t="inlineStr"/>
       <c r="H295" s="4" t="inlineStr"/>
-      <c r="I295" t="inlineStr"/>
       <c r="J295" s="3" t="inlineStr"/>
     </row>
     <row r="296">
@@ -10524,7 +10230,6 @@
       </c>
       <c r="G296" s="3" t="inlineStr"/>
       <c r="H296" s="4" t="inlineStr"/>
-      <c r="I296" t="inlineStr"/>
       <c r="J296" s="3" t="inlineStr"/>
     </row>
     <row r="297">
@@ -10558,7 +10263,6 @@
       </c>
       <c r="G297" s="3" t="inlineStr"/>
       <c r="H297" s="4" t="inlineStr"/>
-      <c r="I297" t="inlineStr"/>
       <c r="J297" s="3" t="inlineStr"/>
     </row>
     <row r="298">
@@ -10592,7 +10296,6 @@
       </c>
       <c r="G298" s="3" t="inlineStr"/>
       <c r="H298" s="4" t="inlineStr"/>
-      <c r="I298" t="inlineStr"/>
       <c r="J298" s="3" t="inlineStr"/>
     </row>
     <row r="299">
@@ -10626,7 +10329,6 @@
       </c>
       <c r="G299" s="3" t="inlineStr"/>
       <c r="H299" s="4" t="inlineStr"/>
-      <c r="I299" t="inlineStr"/>
       <c r="J299" s="3" t="inlineStr"/>
     </row>
     <row r="300">
@@ -10660,7 +10362,6 @@
       </c>
       <c r="G300" s="3" t="inlineStr"/>
       <c r="H300" s="4" t="inlineStr"/>
-      <c r="I300" t="inlineStr"/>
       <c r="J300" s="3" t="inlineStr"/>
     </row>
     <row r="301">
@@ -10694,16 +10395,15 @@
       </c>
       <c r="G301" s="3" t="inlineStr"/>
       <c r="H301" s="4" t="inlineStr"/>
-      <c r="I301" t="inlineStr"/>
       <c r="J301" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <dataValidations count="2">
     <dataValidation sqref="G2:G301" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Nilai tidak dikenal" error="Pilih salah satu nilai dari daftar." type="list">
-      <formula1>"L,L-C1,L-C3,X"</formula1>
+      <formula1>"Yes,Yes-C1,Yes-C3,No"</formula1>
     </dataValidation>
     <dataValidation sqref="J2:J301" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Nilai tidak dikenal" error="Pilih salah satu nilai dari daftar." type="list">
-      <formula1>"L,L-C1,L-C3,X"</formula1>
+      <formula1>"Yes,Yes-C1,Yes-C3,No"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -10738,7 +10438,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -10750,7 +10450,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>L-C1</t>
+          <t>Yes-C1</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -10762,7 +10462,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>L-C3</t>
+          <t>Yes-C3</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -10774,7 +10474,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>No</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">

</xml_diff>